<commit_message>
Readme and License. Backup of eKPIs file in xlsx format.
</commit_message>
<xml_diff>
--- a/Data_Analysis/DemocratizeESG_eKPIS.xlsx
+++ b/Data_Analysis/DemocratizeESG_eKPIS.xlsx
@@ -1,13 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6606eb8fecc814df/Desktop/HKA/MasterThesis/DemocratizeESG/Data_Analysis/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_B248C15BD8A4AE528A4CC9D6200CDF4C8F00095E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA7E61AC-8B41-4382-8F81-8F7CD1ABAD57}"/>
+  <bookViews>
+    <workbookView xWindow="1908" yWindow="-17388" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="industry_agnostic" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="industry_specific" sheetId="2" r:id="rId6"/>
+    <sheet name="industry_agnostic" sheetId="1" r:id="rId1"/>
+    <sheet name="industry_specific" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -671,15 +680,16 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -690,82 +700,35 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF356854"/>
-          <bgColor rgb="FF356854"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
-    <dxf>
-      <font/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF6F8F9"/>
-          <bgColor rgb="FFF6F8F9"/>
-        </patternFill>
-      </fill>
-      <border/>
-    </dxf>
+  <dxfs count="4">
     <dxf>
       <border>
         <left style="thin">
@@ -782,47 +745,67 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="industry_agnostic-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    <tableStyle name="industry_agnostic-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G49" displayName="industry_agnostic_eKPIs" name="industry_agnostic_eKPIs" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="industry_agnostic_eKPIs" displayName="industry_agnostic_eKPIs" ref="A1:G49">
   <tableColumns count="7">
-    <tableColumn name="indicator_id" id="1"/>
-    <tableColumn name="indicator_name" id="2"/>
-    <tableColumn name="indicator_description" id="3"/>
-    <tableColumn name="specific_instructions" id="4"/>
-    <tableColumn name="search_terms" id="5"/>
-    <tableColumn name="is_numeric" id="6"/>
-    <tableColumn name="target_unit" id="7"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="indicator_id"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="indicator_name"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="indicator_description"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="specific_instructions"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="search_terms"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="is_numeric"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="target_unit"/>
   </tableColumns>
-  <tableStyleInfo name="industry_agnostic-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="industry_agnostic-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1012,26 +995,29 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G49"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="27.25"/>
-    <col customWidth="1" min="2" max="2" width="31.13"/>
-    <col customWidth="1" min="3" max="3" width="33.5"/>
-    <col customWidth="1" min="4" max="4" width="20.75"/>
-    <col customWidth="1" min="5" max="5" width="15.5"/>
-    <col customWidth="1" min="6" max="6" width="16.75"/>
-    <col customWidth="1" min="7" max="7" width="26.0"/>
+    <col min="1" max="1" width="27.265625" customWidth="1"/>
+    <col min="2" max="2" width="31.1328125" customWidth="1"/>
+    <col min="3" max="3" width="33.46484375" customWidth="1"/>
+    <col min="4" max="4" width="20.73046875" customWidth="1"/>
+    <col min="5" max="5" width="15.46484375" customWidth="1"/>
+    <col min="6" max="6" width="16.73046875" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1">
+    <row r="1" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1054,7 +1040,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
+    <row r="2" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1070,14 +1056,14 @@
       <c r="E2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G2" s="3" t="s">
+      <c r="F2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" ht="22.5" customHeight="1">
+    <row r="3" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>14</v>
       </c>
@@ -1093,523 +1079,523 @@
       <c r="E3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="3" t="s">
+      <c r="F3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4" t="s">
+      <c r="D5" s="2"/>
+      <c r="E5" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4" t="s">
+      <c r="D6" s="2"/>
+      <c r="E6" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="5" t="s">
+      <c r="F8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="4" t="s">
+    <row r="9" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G9" s="5" t="s">
+      <c r="F9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F10" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="5" t="s">
+      <c r="F10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4" t="s">
+      <c r="D11" s="2"/>
+      <c r="E11" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G11" s="5" t="s">
+      <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="4" t="s">
+    <row r="12" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G12" s="5" t="s">
+      <c r="F12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G13" s="5" t="s">
+      <c r="F13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="2" t="s">
         <v>63</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E14" s="4"/>
-      <c r="F14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G14" s="5" t="s">
+      <c r="E14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="4" t="s">
+    <row r="15" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="2" t="s">
         <v>67</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G15" s="5" t="s">
+      <c r="F15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="4" t="s">
+    <row r="16" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="2" t="s">
         <v>73</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="5" t="s">
+      <c r="F16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="4" t="s">
+    <row r="17" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="2" t="s">
         <v>78</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4" t="s">
+      <c r="D17" s="2"/>
+      <c r="E17" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="F17" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G17" s="5" t="s">
+      <c r="F17" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="4" t="s">
+    <row r="18" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F18" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G18" s="5" t="s">
+      <c r="F18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="19" ht="22.5" customHeight="1">
-      <c r="A19" s="4" t="s">
+    <row r="19" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="F19" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G19" s="5" t="s">
+      <c r="F19" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="20" ht="22.5" customHeight="1">
-      <c r="A20" s="4" t="s">
+    <row r="20" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="2" t="s">
         <v>93</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="F20" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G20" s="5" t="s">
+      <c r="F20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="21" ht="22.5" customHeight="1">
-      <c r="A21" s="4" t="s">
+    <row r="21" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="F21" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G21" s="5" t="s">
+      <c r="F21" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G21" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="22" ht="22.5" customHeight="1">
-      <c r="A22" s="4" t="s">
+    <row r="22" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="2" t="s">
         <v>103</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="F22" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G22" s="5" t="s">
+      <c r="F22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="23" ht="22.5" customHeight="1">
-      <c r="A23" s="4" t="s">
+    <row r="23" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
         <v>107</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="F23" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G23" s="5" t="s">
+      <c r="F23" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="24" ht="22.5" customHeight="1">
-      <c r="A24" s="4" t="s">
+    <row r="24" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="2" t="s">
         <v>113</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F24" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G24" s="5" t="s">
+      <c r="F24" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="25" ht="22.5" customHeight="1">
-      <c r="A25" s="4" t="s">
+    <row r="25" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="2" t="s">
         <v>116</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="2" t="s">
         <v>118</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="E25" s="4" t="s">
+      <c r="E25" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="F25" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G25" s="5" t="s">
+      <c r="F25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="26" ht="22.5" customHeight="1">
-      <c r="A26" s="4" t="s">
+    <row r="26" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="2" t="s">
         <v>121</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="2" t="s">
         <v>123</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G26" s="5" t="s">
+      <c r="E26" s="2"/>
+      <c r="F26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="27" ht="22.5" customHeight="1">
-      <c r="A27" s="4" t="s">
+    <row r="27" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="2" t="s">
         <v>126</v>
       </c>
       <c r="B27" s="2" t="s">
@@ -1621,16 +1607,16 @@
       <c r="D27" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="F27" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G27" s="6"/>
-    </row>
-    <row r="28" ht="22.5" customHeight="1">
-      <c r="A28" s="4" t="s">
+      <c r="G27" s="2"/>
+    </row>
+    <row r="28" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="2" t="s">
         <v>131</v>
       </c>
       <c r="B28" s="2" t="s">
@@ -1642,16 +1628,16 @@
       <c r="D28" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F28" s="5" t="s">
+      <c r="F28" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G28" s="6"/>
-    </row>
-    <row r="29" ht="22.5" customHeight="1">
-      <c r="A29" s="4" t="s">
+      <c r="G28" s="2"/>
+    </row>
+    <row r="29" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="2" t="s">
         <v>136</v>
       </c>
       <c r="B29" s="2" t="s">
@@ -1663,14 +1649,14 @@
       <c r="D29" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="5" t="s">
+      <c r="E29" s="2"/>
+      <c r="F29" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G29" s="6"/>
-    </row>
-    <row r="30" ht="22.5" customHeight="1">
-      <c r="A30" s="4" t="s">
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="2" t="s">
         <v>140</v>
       </c>
       <c r="B30" s="2" t="s">
@@ -1682,14 +1668,14 @@
       <c r="D30" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E30" s="4"/>
-      <c r="F30" s="5" t="s">
+      <c r="E30" s="2"/>
+      <c r="F30" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G30" s="6"/>
-    </row>
-    <row r="31" ht="22.5" customHeight="1">
-      <c r="A31" s="4" t="s">
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="2" t="s">
         <v>144</v>
       </c>
       <c r="B31" s="2" t="s">
@@ -1701,16 +1687,16 @@
       <c r="D31" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E31" s="4" t="s">
+      <c r="E31" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F31" s="5" t="s">
+      <c r="F31" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G31" s="6"/>
-    </row>
-    <row r="32" ht="22.5" customHeight="1">
-      <c r="A32" s="4" t="s">
+      <c r="G31" s="2"/>
+    </row>
+    <row r="32" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="2" t="s">
         <v>147</v>
       </c>
       <c r="B32" s="2" t="s">
@@ -1722,14 +1708,14 @@
       <c r="D32" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="5" t="s">
+      <c r="E32" s="2"/>
+      <c r="F32" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G32" s="6"/>
-    </row>
-    <row r="33" ht="22.5" customHeight="1">
-      <c r="A33" s="4" t="s">
+      <c r="G32" s="2"/>
+    </row>
+    <row r="33" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>150</v>
       </c>
       <c r="B33" s="2" t="s">
@@ -1741,14 +1727,14 @@
       <c r="D33" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="5" t="s">
+      <c r="E33" s="2"/>
+      <c r="F33" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G33" s="6"/>
-    </row>
-    <row r="34" ht="22.5" customHeight="1">
-      <c r="A34" s="4" t="s">
+      <c r="G33" s="2"/>
+    </row>
+    <row r="34" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="2" t="s">
         <v>152</v>
       </c>
       <c r="B34" s="2" t="s">
@@ -1760,14 +1746,14 @@
       <c r="D34" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="5" t="s">
+      <c r="E34" s="2"/>
+      <c r="F34" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G34" s="6"/>
-    </row>
-    <row r="35" ht="22.5" customHeight="1">
-      <c r="A35" s="4" t="s">
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="2" t="s">
         <v>154</v>
       </c>
       <c r="B35" s="2" t="s">
@@ -1779,14 +1765,14 @@
       <c r="D35" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="5" t="s">
+      <c r="E35" s="2"/>
+      <c r="F35" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G35" s="6"/>
-    </row>
-    <row r="36" ht="22.5" customHeight="1">
-      <c r="A36" s="4" t="s">
+      <c r="G35" s="2"/>
+    </row>
+    <row r="36" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="2" t="s">
         <v>158</v>
       </c>
       <c r="B36" s="2" t="s">
@@ -1798,14 +1784,14 @@
       <c r="D36" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E36" s="4"/>
-      <c r="F36" s="5" t="s">
+      <c r="E36" s="2"/>
+      <c r="F36" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G36" s="6"/>
-    </row>
-    <row r="37" ht="22.5" customHeight="1">
-      <c r="A37" s="4" t="s">
+      <c r="G36" s="2"/>
+    </row>
+    <row r="37" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="2" t="s">
         <v>162</v>
       </c>
       <c r="B37" s="2" t="s">
@@ -1817,14 +1803,14 @@
       <c r="D37" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="E37" s="4"/>
-      <c r="F37" s="5" t="s">
+      <c r="E37" s="2"/>
+      <c r="F37" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G37" s="6"/>
-    </row>
-    <row r="38" ht="22.5" customHeight="1">
-      <c r="A38" s="4" t="s">
+      <c r="G37" s="2"/>
+    </row>
+    <row r="38" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
         <v>165</v>
       </c>
       <c r="B38" s="2" t="s">
@@ -1836,14 +1822,14 @@
       <c r="D38" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E38" s="4"/>
-      <c r="F38" s="5" t="s">
+      <c r="E38" s="2"/>
+      <c r="F38" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G38" s="6"/>
-    </row>
-    <row r="39" ht="22.5" customHeight="1">
-      <c r="A39" s="4" t="s">
+      <c r="G38" s="2"/>
+    </row>
+    <row r="39" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
         <v>169</v>
       </c>
       <c r="B39" s="2" t="s">
@@ -1855,14 +1841,14 @@
       <c r="D39" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="E39" s="4"/>
-      <c r="F39" s="5" t="s">
+      <c r="E39" s="2"/>
+      <c r="F39" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G39" s="6"/>
-    </row>
-    <row r="40" ht="22.5" customHeight="1">
-      <c r="A40" s="4" t="s">
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
         <v>172</v>
       </c>
       <c r="B40" s="2" t="s">
@@ -1874,16 +1860,16 @@
       <c r="D40" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="E40" s="4" t="s">
+      <c r="E40" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="F40" s="5" t="s">
+      <c r="F40" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G40" s="6"/>
-    </row>
-    <row r="41" ht="22.5" customHeight="1">
-      <c r="A41" s="4" t="s">
+      <c r="G40" s="2"/>
+    </row>
+    <row r="41" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
         <v>177</v>
       </c>
       <c r="B41" s="2" t="s">
@@ -1893,16 +1879,16 @@
         <v>179</v>
       </c>
       <c r="D41" s="2"/>
-      <c r="E41" s="4" t="s">
+      <c r="E41" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="F41" s="5" t="s">
+      <c r="F41" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G41" s="6"/>
-    </row>
-    <row r="42" ht="22.5" customHeight="1">
-      <c r="A42" s="4" t="s">
+      <c r="G41" s="2"/>
+    </row>
+    <row r="42" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
         <v>181</v>
       </c>
       <c r="B42" s="2" t="s">
@@ -1912,18 +1898,18 @@
         <v>183</v>
       </c>
       <c r="D42" s="2"/>
-      <c r="E42" s="4" t="s">
+      <c r="E42" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F42" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G42" s="5" t="s">
+      <c r="F42" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G42" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="43" ht="22.5" customHeight="1">
-      <c r="A43" s="4" t="s">
+    <row r="43" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
         <v>185</v>
       </c>
       <c r="B43" s="2" t="s">
@@ -1935,16 +1921,16 @@
       <c r="D43" s="2" t="s">
         <v>188</v>
       </c>
-      <c r="E43" s="4" t="s">
+      <c r="E43" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="F43" s="5" t="s">
+      <c r="F43" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G43" s="6"/>
-    </row>
-    <row r="44" ht="22.5" customHeight="1">
-      <c r="A44" s="4" t="s">
+      <c r="G43" s="2"/>
+    </row>
+    <row r="44" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
         <v>190</v>
       </c>
       <c r="B44" s="2" t="s">
@@ -1956,16 +1942,16 @@
       <c r="D44" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="E44" s="4" t="s">
+      <c r="E44" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="F44" s="5" t="s">
+      <c r="F44" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G44" s="6"/>
-    </row>
-    <row r="45" ht="22.5" customHeight="1">
-      <c r="A45" s="4" t="s">
+      <c r="G44" s="2"/>
+    </row>
+    <row r="45" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="2" t="s">
         <v>195</v>
       </c>
       <c r="B45" s="2" t="s">
@@ -1975,16 +1961,16 @@
         <v>197</v>
       </c>
       <c r="D45" s="2"/>
-      <c r="E45" s="4" t="s">
+      <c r="E45" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="F45" s="5" t="s">
+      <c r="F45" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G45" s="6"/>
-    </row>
-    <row r="46" ht="22.5" customHeight="1">
-      <c r="A46" s="4" t="s">
+      <c r="G45" s="2"/>
+    </row>
+    <row r="46" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="2" t="s">
         <v>199</v>
       </c>
       <c r="B46" s="2" t="s">
@@ -1994,16 +1980,16 @@
         <v>201</v>
       </c>
       <c r="D46" s="2"/>
-      <c r="E46" s="4" t="s">
+      <c r="E46" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="F46" s="5" t="s">
+      <c r="F46" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G46" s="6"/>
-    </row>
-    <row r="47" ht="22.5" customHeight="1">
-      <c r="A47" s="4" t="s">
+      <c r="G46" s="2"/>
+    </row>
+    <row r="47" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="2" t="s">
         <v>203</v>
       </c>
       <c r="B47" s="2" t="s">
@@ -2013,18 +1999,18 @@
         <v>205</v>
       </c>
       <c r="D47" s="2"/>
-      <c r="E47" s="4" t="s">
+      <c r="E47" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="F47" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G47" s="5" t="s">
+      <c r="F47" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G47" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="48" ht="22.5" customHeight="1">
-      <c r="A48" s="4" t="s">
+    <row r="48" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
         <v>207</v>
       </c>
       <c r="B48" s="2" t="s">
@@ -2036,18 +2022,18 @@
       <c r="D48" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="E48" s="4" t="s">
+      <c r="E48" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="F48" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G48" s="5" t="s">
+      <c r="F48" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="49" ht="22.5" customHeight="1">
-      <c r="A49" s="4" t="s">
+    <row r="49" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
         <v>212</v>
       </c>
       <c r="B49" s="2" t="s">
@@ -2059,63 +2045,64 @@
       <c r="D49" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E49" s="4" t="s">
+      <c r="E49" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="F49" s="5" t="s">
+      <c r="F49" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="G49" s="6"/>
+      <c r="G49" s="2"/>
     </row>
   </sheetData>
-  <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="G2:G49">
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G49" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"tonnes,thousand cubic meters,square meters,million tonnes of CO2,million cubic meters,l/100km,km,kg/ton,GWh,GJ,gCO₂/km,billion euros,bbl"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F49">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F49" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr defaultColWidth="12.59765625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col customWidth="1" min="3" max="3" width="16.25"/>
-    <col customWidth="1" min="4" max="4" width="17.0"/>
-    <col customWidth="1" min="5" max="5" width="14.5"/>
+    <col min="3" max="3" width="16.265625" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="24.3984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>